<commit_message>
fix: replace example GL workbook with corrected sign direction
</commit_message>
<xml_diff>
--- a/examples/gl_data.xlsx
+++ b/examples/gl_data.xlsx
@@ -1,13 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raysa\OneDrive - CHIPMUNK ROBOTICS LIMITED LIABILITY CO\Desktop\Technology Demo\Bank Recon Skill\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB5B09E-5FCD-4ECE-A350-1BECDB26E4CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="GL Data" sheetId="1" r:id="rId4"/>
+    <sheet name="GL Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="sOrPa2gKKw69CJkBbRQ02cVFFiXeDXyM9mQftAmSwiU="/>
     </ext>
@@ -885,15 +905,16 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
@@ -904,34 +925,43 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1121,20 +1151,23 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C1000"/>
+  <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="10.0"/>
-    <col customWidth="1" min="2" max="2" width="9.0"/>
-    <col customWidth="1" min="3" max="3" width="92.14"/>
-    <col customWidth="1" min="4" max="26" width="8.71"/>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="9.5" customWidth="1"/>
+    <col min="3" max="3" width="92.09765625" customWidth="1"/>
+    <col min="4" max="26" width="8.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1145,3006 +1178,3006 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1">
-        <v>-6505.99</v>
+        <v>6505.99</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1">
-        <v>-2635.29</v>
+        <v>2635.29</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>3528.92</v>
+        <v>-3528.92</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="1">
-        <v>-12770.47</v>
+        <v>12770.47</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="1">
-        <v>-48.99</v>
+        <v>48.99</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="1">
-        <v>-8220.15</v>
+        <v>8220.15</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B8" s="1">
-        <v>-1210.8</v>
+        <v>1210.8</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="1">
-        <v>1390.13</v>
+        <v>-1390.13</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="1">
-        <v>2834.59</v>
+        <v>-2834.59</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B11" s="1">
-        <v>4331.3</v>
+        <v>-4331.3</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="1">
-        <v>5715.95</v>
+        <v>-5715.95</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="1">
-        <v>7382.09</v>
+        <v>-7382.09</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="1">
-        <v>-445.28</v>
+        <v>445.28</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B15" s="1">
-        <v>5860.78</v>
+        <v>-5860.78</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B16" s="1">
-        <v>5675.43</v>
+        <v>-5675.43</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B17" s="1">
-        <v>1112.07</v>
+        <v>-1112.07</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B18" s="1">
-        <v>2328.15</v>
+        <v>-2328.15</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B19" s="1">
-        <v>-3420.7</v>
+        <v>3420.7</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B20" s="1">
-        <v>-65.48</v>
+        <v>65.48</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B21" s="1">
-        <v>-14484.4</v>
+        <v>14484.4</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B22" s="1">
-        <v>-12782.98</v>
+        <v>12782.98</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B23" s="1">
-        <v>-103.77</v>
+        <v>103.77</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B24" s="1">
-        <v>-15.0</v>
+        <v>15</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B25" s="1">
-        <v>-26698.04</v>
+        <v>26698.04</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B26" s="1">
-        <v>-2365.75</v>
+        <v>2365.75</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B27" s="1">
-        <v>-3135.93</v>
+        <v>3135.93</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B28" s="1">
-        <v>-41.01</v>
+        <v>41.01</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B29" s="1">
-        <v>-17.42</v>
+        <v>17.420000000000002</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B30" s="1">
-        <v>-15.41</v>
+        <v>15.41</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B31" s="1">
-        <v>1202.37</v>
+        <v>-1202.3699999999999</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B32" s="1">
-        <v>1482.81</v>
+        <v>-1482.81</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B33" s="1">
-        <v>4214.41</v>
+        <v>-4214.41</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
+    <row r="34" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B34" s="1">
-        <v>4568.69</v>
+        <v>-4568.6899999999996</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
+    <row r="35" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B35" s="1">
-        <v>-19.45</v>
+        <v>19.45</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
+    <row r="36" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B36" s="1">
-        <v>930.92</v>
+        <v>-930.92</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B37" s="1">
-        <v>4676.54</v>
+        <v>-4676.54</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
+    <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B38" s="1">
-        <v>4712.08</v>
+        <v>-4712.08</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="39" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B39" s="1">
-        <v>4086.46</v>
+        <v>-4086.46</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B40" s="1">
-        <v>-2435.88</v>
+        <v>2435.88</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B41" s="1">
-        <v>2470.27</v>
+        <v>-2470.27</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
+    <row r="42" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B42" s="1">
-        <v>-1963.77</v>
+        <v>1963.77</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
+    <row r="43" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B43" s="1">
-        <v>-1662.16</v>
+        <v>1662.16</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B44" s="1">
-        <v>-587.64</v>
+        <v>587.64</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B45" s="1">
-        <v>778.62</v>
+        <v>-778.62</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
+    <row r="46" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B46" s="1">
-        <v>1184.75</v>
+        <v>-1184.75</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
+    <row r="47" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B47" s="1">
-        <v>-7424.24</v>
+        <v>7424.24</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="48" ht="15.75" customHeight="1">
+    <row r="48" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B48" s="1">
-        <v>-11087.46</v>
+        <v>11087.46</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
+    <row r="49" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B49" s="1">
-        <v>-15.0</v>
+        <v>15</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>72</v>
       </c>
       <c r="B50" s="1">
-        <v>-1382.97</v>
+        <v>1382.97</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B51" s="1">
-        <v>-9223.06</v>
+        <v>9223.06</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
+    <row r="52" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B52" s="1">
-        <v>-107.2</v>
+        <v>107.2</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
+    <row r="53" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B53" s="1">
-        <v>15632.86</v>
+        <v>-15632.86</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="54" ht="15.75" customHeight="1">
+    <row r="54" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B54" s="1">
-        <v>4032.82</v>
+        <v>-4032.82</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="55" ht="15.75" customHeight="1">
+    <row r="55" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B55" s="1">
-        <v>8801.55</v>
+        <v>-8801.5499999999993</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="56" ht="15.75" customHeight="1">
+    <row r="56" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>83</v>
       </c>
       <c r="B56" s="1">
-        <v>-209.57</v>
+        <v>209.57</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="57" ht="15.75" customHeight="1">
+    <row r="57" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>85</v>
       </c>
       <c r="B57" s="1">
-        <v>-367.44</v>
+        <v>367.44</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="58" ht="15.75" customHeight="1">
+    <row r="58" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B58" s="1">
-        <v>-2166.62</v>
+        <v>2166.62</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="59" ht="15.75" customHeight="1">
+    <row r="59" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B59" s="1">
-        <v>-1268.09</v>
+        <v>1268.0899999999999</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="60" ht="15.75" customHeight="1">
+    <row r="60" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B60" s="1">
-        <v>-246.01</v>
+        <v>246.01</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="61" ht="15.75" customHeight="1">
+    <row r="61" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B61" s="1">
-        <v>-127.42</v>
+        <v>127.42</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="62" ht="15.75" customHeight="1">
+    <row r="62" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B62" s="1">
-        <v>-4564.85</v>
+        <v>4564.8500000000004</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="63" ht="15.75" customHeight="1">
+    <row r="63" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B63" s="1">
-        <v>8481.46</v>
+        <v>-8481.4599999999991</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="64" ht="15.75" customHeight="1">
+    <row r="64" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>95</v>
       </c>
       <c r="B64" s="1">
-        <v>-683.27</v>
+        <v>683.27</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="65" ht="15.75" customHeight="1">
+    <row r="65" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>95</v>
       </c>
       <c r="B65" s="1">
-        <v>-153.45</v>
+        <v>153.44999999999999</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="66" ht="15.75" customHeight="1">
+    <row r="66" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B66" s="1">
-        <v>-122.8</v>
+        <v>122.8</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="67" ht="15.75" customHeight="1">
+    <row r="67" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B67" s="1">
-        <v>-44.21</v>
+        <v>44.21</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="68" ht="15.75" customHeight="1">
+    <row r="68" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B68" s="1">
-        <v>1179.53</v>
+        <v>-1179.53</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="69" ht="15.75" customHeight="1">
+    <row r="69" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B69" s="1">
-        <v>3032.24</v>
+        <v>-3032.24</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="70" ht="15.75" customHeight="1">
+    <row r="70" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B70" s="1">
-        <v>3291.06</v>
+        <v>-3291.06</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="71" ht="15.75" customHeight="1">
+    <row r="71" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B71" s="1">
-        <v>8240.63</v>
+        <v>-8240.6299999999992</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="72" ht="15.75" customHeight="1">
+    <row r="72" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>105</v>
       </c>
       <c r="B72" s="1">
-        <v>-994.4</v>
+        <v>994.4</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="73" ht="15.75" customHeight="1">
+    <row r="73" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>105</v>
       </c>
       <c r="B73" s="1">
-        <v>3075.79</v>
+        <v>-3075.79</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="74" ht="15.75" customHeight="1">
+    <row r="74" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>108</v>
       </c>
       <c r="B74" s="1">
-        <v>938.06</v>
+        <v>-938.06</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="75" ht="15.75" customHeight="1">
+    <row r="75" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>110</v>
       </c>
       <c r="B75" s="1">
-        <v>-723.2</v>
+        <v>723.2</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="76" ht="15.75" customHeight="1">
+    <row r="76" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>112</v>
       </c>
       <c r="B76" s="1">
-        <v>-1377.86</v>
+        <v>1377.86</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="77" ht="15.75" customHeight="1">
+    <row r="77" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B77" s="1">
-        <v>-9706.14</v>
+        <v>9706.14</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="78" ht="15.75" customHeight="1">
+    <row r="78" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B78" s="1">
-        <v>-7602.67</v>
+        <v>7602.67</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="79" ht="15.75" customHeight="1">
+    <row r="79" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B79" s="1">
-        <v>-2019.35</v>
+        <v>2019.35</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="80" ht="15.75" customHeight="1">
+    <row r="80" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B80" s="1">
-        <v>1316.01</v>
+        <v>-1316.01</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="81" ht="15.75" customHeight="1">
+    <row r="81" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B81" s="1">
-        <v>4322.15</v>
+        <v>-4322.1499999999996</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="82" ht="15.75" customHeight="1">
+    <row r="82" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B82" s="1">
-        <v>9097.82</v>
+        <v>-9097.82</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="83" ht="15.75" customHeight="1">
+    <row r="83" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B83" s="1">
-        <v>-14210.57</v>
+        <v>14210.57</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="84" ht="15.75" customHeight="1">
+    <row r="84" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B84" s="1">
-        <v>20.0</v>
+        <v>-20</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="85" ht="15.75" customHeight="1">
+    <row r="85" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>124</v>
       </c>
       <c r="B85" s="1">
-        <v>-1733.51</v>
+        <v>1733.51</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="86" ht="15.75" customHeight="1">
+    <row r="86" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>124</v>
       </c>
       <c r="B86" s="1">
-        <v>-904.4</v>
+        <v>904.4</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="87" ht="15.75" customHeight="1">
+    <row r="87" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>124</v>
       </c>
       <c r="B87" s="1">
-        <v>-767.06</v>
+        <v>767.06</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="88" ht="15.75" customHeight="1">
+    <row r="88" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>128</v>
       </c>
       <c r="B88" s="1">
-        <v>-349.05</v>
+        <v>349.05</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="89" ht="15.75" customHeight="1">
+    <row r="89" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>130</v>
       </c>
       <c r="B89" s="1">
-        <v>-1727.56</v>
+        <v>1727.56</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="90" ht="15.75" customHeight="1">
+    <row r="90" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B90" s="1">
-        <v>99.57</v>
+        <v>-99.57</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="91" ht="15.75" customHeight="1">
+    <row r="91" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B91" s="1">
-        <v>550.97</v>
+        <v>-550.97</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="92" ht="15.75" customHeight="1">
+    <row r="92" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B92" s="1">
-        <v>2875.13</v>
+        <v>-2875.13</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="93" ht="15.75" customHeight="1">
+    <row r="93" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B93" s="1">
-        <v>2889.25</v>
+        <v>-2889.25</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="94" ht="15.75" customHeight="1">
+    <row r="94" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>137</v>
       </c>
       <c r="B94" s="1">
-        <v>-1653.91</v>
+        <v>1653.91</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="95" ht="15.75" customHeight="1">
+    <row r="95" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>137</v>
       </c>
       <c r="B95" s="1">
-        <v>1698.48</v>
+        <v>-1698.48</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="96" ht="15.75" customHeight="1">
+    <row r="96" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B96" s="1">
-        <v>-9240.58</v>
+        <v>9240.58</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="97" ht="15.75" customHeight="1">
+    <row r="97" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B97" s="1">
-        <v>-6585.18</v>
+        <v>6585.18</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="98" ht="15.75" customHeight="1">
+    <row r="98" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B98" s="1">
-        <v>-1788.37</v>
+        <v>1788.37</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="99" ht="15.75" customHeight="1">
+    <row r="99" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B99" s="1">
-        <v>585.61</v>
+        <v>-585.61</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="100" ht="15.75" customHeight="1">
+    <row r="100" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B100" s="1">
-        <v>1925.58</v>
+        <v>-1925.58</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="101" ht="15.75" customHeight="1">
+    <row r="101" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>146</v>
       </c>
       <c r="B101" s="1">
-        <v>-420.72</v>
+        <v>420.72</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="102" ht="15.75" customHeight="1">
+    <row r="102" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>148</v>
       </c>
       <c r="B102" s="1">
-        <v>3413.17</v>
+        <v>-3413.17</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="103" ht="15.75" customHeight="1">
+    <row r="103" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B103" s="1">
-        <v>-15.0</v>
+        <v>15</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="104" ht="15.75" customHeight="1">
+    <row r="104" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B104" s="1">
-        <v>-3511.03</v>
+        <v>3511.03</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="105" ht="15.75" customHeight="1">
+    <row r="105" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B105" s="1">
-        <v>-488.64</v>
+        <v>488.64</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="106" ht="15.75" customHeight="1">
+    <row r="106" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B106" s="1">
-        <v>-379.45</v>
+        <v>379.45</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="107" ht="15.75" customHeight="1">
+    <row r="107" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B107" s="1">
-        <v>4051.6</v>
+        <v>-4051.6</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="108" ht="15.75" customHeight="1">
+    <row r="108" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>157</v>
       </c>
       <c r="B108" s="1">
-        <v>-293.98</v>
+        <v>293.98</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="109" ht="15.75" customHeight="1">
+    <row r="109" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>157</v>
       </c>
       <c r="B109" s="1">
-        <v>982.51</v>
+        <v>-982.51</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="110" ht="15.75" customHeight="1">
+    <row r="110" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>157</v>
       </c>
       <c r="B110" s="1">
-        <v>1057.48</v>
+        <v>-1057.48</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="111" ht="15.75" customHeight="1">
+    <row r="111" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>157</v>
       </c>
       <c r="B111" s="1">
-        <v>5626.38</v>
+        <v>-5626.38</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="112" ht="15.75" customHeight="1">
+    <row r="112" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B112" s="1">
-        <v>-587.64</v>
+        <v>587.64</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="113" ht="15.75" customHeight="1">
+    <row r="113" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>164</v>
       </c>
       <c r="B113" s="1">
-        <v>-199.54</v>
+        <v>199.54</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="114" ht="15.75" customHeight="1">
+    <row r="114" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>166</v>
       </c>
       <c r="B114" s="1">
-        <v>-353.4</v>
+        <v>353.4</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="115" ht="15.75" customHeight="1">
+    <row r="115" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>166</v>
       </c>
       <c r="B115" s="1">
-        <v>357.51</v>
+        <v>-357.51</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="116" ht="15.75" customHeight="1">
+    <row r="116" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>166</v>
       </c>
       <c r="B116" s="1">
-        <v>2416.63</v>
+        <v>-2416.63</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="117" ht="15.75" customHeight="1">
+    <row r="117" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>166</v>
       </c>
       <c r="B117" s="1">
-        <v>16203.9</v>
+        <v>-16203.9</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="118" ht="15.75" customHeight="1">
+    <row r="118" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>171</v>
       </c>
       <c r="B118" s="1">
-        <v>20.0</v>
+        <v>-20</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="119" ht="15.75" customHeight="1">
+    <row r="119" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>171</v>
       </c>
       <c r="B119" s="1">
-        <v>4016.88</v>
+        <v>-4016.88</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="120" ht="15.75" customHeight="1">
+    <row r="120" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>174</v>
       </c>
       <c r="B120" s="1">
-        <v>-944.81</v>
+        <v>944.81</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="121" ht="15.75" customHeight="1">
+    <row r="121" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>176</v>
       </c>
       <c r="B121" s="1">
-        <v>-313.72</v>
+        <v>313.72000000000003</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="122" ht="15.75" customHeight="1">
+    <row r="122" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>176</v>
       </c>
       <c r="B122" s="1">
-        <v>-72.42</v>
+        <v>72.42</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="123" ht="15.75" customHeight="1">
+    <row r="123" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>179</v>
       </c>
       <c r="B123" s="1">
-        <v>-66.01</v>
+        <v>66.010000000000005</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="124" ht="15.75" customHeight="1">
+    <row r="124" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>181</v>
       </c>
       <c r="B124" s="1">
-        <v>8014.95</v>
+        <v>-8014.95</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="125" ht="15.75" customHeight="1">
+    <row r="125" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>183</v>
       </c>
       <c r="B125" s="1">
-        <v>1901.02</v>
+        <v>-1901.02</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="126" ht="15.75" customHeight="1">
+    <row r="126" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>183</v>
       </c>
       <c r="B126" s="1">
-        <v>5806.69</v>
+        <v>-5806.69</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="127" ht="15.75" customHeight="1">
+    <row r="127" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>186</v>
       </c>
       <c r="B127" s="1">
-        <v>-4039.51</v>
+        <v>4039.51</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="128" ht="15.75" customHeight="1">
+    <row r="128" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>186</v>
       </c>
       <c r="B128" s="1">
-        <v>-2690.66</v>
+        <v>2690.66</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="129" ht="15.75" customHeight="1">
+    <row r="129" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>186</v>
       </c>
       <c r="B129" s="1">
-        <v>-1125.9</v>
+        <v>1125.9000000000001</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="130" ht="15.75" customHeight="1">
+    <row r="130" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>186</v>
       </c>
       <c r="B130" s="1">
-        <v>-720.22</v>
+        <v>720.22</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="131" ht="15.75" customHeight="1">
+    <row r="131" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>186</v>
       </c>
       <c r="B131" s="1">
-        <v>-513.61</v>
+        <v>513.61</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="132" ht="15.75" customHeight="1">
+    <row r="132" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>186</v>
       </c>
       <c r="B132" s="1">
-        <v>5948.85</v>
+        <v>-5948.85</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="133" ht="15.75" customHeight="1">
+    <row r="133" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>186</v>
       </c>
       <c r="B133" s="1">
-        <v>8156.96</v>
+        <v>-8156.96</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="134" ht="15.75" customHeight="1">
+    <row r="134" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>194</v>
       </c>
       <c r="B134" s="1">
-        <v>-383.36</v>
+        <v>383.36</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="135" ht="15.75" customHeight="1">
+    <row r="135" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>196</v>
       </c>
       <c r="B135" s="1">
-        <v>-1304.65</v>
+        <v>1304.6500000000001</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="136" ht="15.75" customHeight="1">
+    <row r="136" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>198</v>
       </c>
       <c r="B136" s="1">
-        <v>-15.0</v>
+        <v>15</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="137" ht="15.75" customHeight="1">
+    <row r="137" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>200</v>
       </c>
       <c r="B137" s="1">
-        <v>-731.52</v>
+        <v>731.52</v>
       </c>
       <c r="C137" s="1" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="138" ht="15.75" customHeight="1">
+    <row r="138" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>200</v>
       </c>
       <c r="B138" s="1">
-        <v>894.47</v>
+        <v>-894.47</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="139" ht="15.75" customHeight="1">
+    <row r="139" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>200</v>
       </c>
       <c r="B139" s="1">
-        <v>8013.05</v>
+        <v>-8013.05</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="140" ht="15.75" customHeight="1">
+    <row r="140" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>204</v>
       </c>
       <c r="B140" s="1">
-        <v>-6587.69</v>
+        <v>6587.69</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="141" ht="15.75" customHeight="1">
+    <row r="141" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>204</v>
       </c>
       <c r="B141" s="1">
-        <v>-1387.59</v>
+        <v>1387.59</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="142" ht="15.75" customHeight="1">
+    <row r="142" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>204</v>
       </c>
       <c r="B142" s="1">
-        <v>4629.55</v>
+        <v>-4629.55</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="143" ht="15.75" customHeight="1">
+    <row r="143" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>208</v>
       </c>
       <c r="B143" s="1">
-        <v>1428.62</v>
+        <v>-1428.62</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="144" ht="15.75" customHeight="1">
+    <row r="144" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>208</v>
       </c>
       <c r="B144" s="1">
-        <v>3527.41</v>
+        <v>-3527.41</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="145" ht="15.75" customHeight="1">
+    <row r="145" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>211</v>
       </c>
       <c r="B145" s="1">
-        <v>-4036.4</v>
+        <v>4036.4</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="146" ht="15.75" customHeight="1">
+    <row r="146" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>211</v>
       </c>
       <c r="B146" s="1">
-        <v>-1702.19</v>
+        <v>1702.19</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="147" ht="15.75" customHeight="1">
+    <row r="147" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>211</v>
       </c>
       <c r="B147" s="1">
-        <v>-664.44</v>
+        <v>664.44</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="148" ht="15.75" customHeight="1">
+    <row r="148" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>215</v>
       </c>
       <c r="B148" s="1">
-        <v>553.11</v>
+        <v>-553.11</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="149" ht="15.75" customHeight="1">
+    <row r="149" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>217</v>
       </c>
       <c r="B149" s="1">
-        <v>-7104.29</v>
+        <v>7104.29</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="150" ht="15.75" customHeight="1">
+    <row r="150" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>217</v>
       </c>
       <c r="B150" s="1">
-        <v>-6064.27</v>
+        <v>6064.27</v>
       </c>
       <c r="C150" s="1" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="151" ht="15.75" customHeight="1">
+    <row r="151" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>217</v>
       </c>
       <c r="B151" s="1">
-        <v>-2018.9</v>
+        <v>2018.9</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="152" ht="15.75" customHeight="1">
+    <row r="152" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>217</v>
       </c>
       <c r="B152" s="1">
-        <v>2740.65</v>
+        <v>-2740.65</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="153" ht="15.75" customHeight="1">
+    <row r="153" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>217</v>
       </c>
       <c r="B153" s="1">
-        <v>2884.28</v>
+        <v>-2884.28</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="154" ht="15.75" customHeight="1">
+    <row r="154" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>217</v>
       </c>
       <c r="B154" s="1">
-        <v>3509.64</v>
+        <v>-3509.64</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="155" ht="15.75" customHeight="1">
+    <row r="155" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>217</v>
       </c>
       <c r="B155" s="1">
-        <v>6490.7</v>
+        <v>-6490.7</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="156" ht="15.75" customHeight="1">
+    <row r="156" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>225</v>
       </c>
       <c r="B156" s="1">
-        <v>-5322.31</v>
+        <v>5322.31</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="157" ht="15.75" customHeight="1">
+    <row r="157" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B157" s="1">
-        <v>-898.82</v>
+        <v>898.82</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="158" ht="15.75" customHeight="1">
+    <row r="158" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B158" s="1">
-        <v>-226.22</v>
+        <v>226.22</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="159" ht="15.75" customHeight="1">
+    <row r="159" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B159" s="1">
-        <v>662.25</v>
+        <v>-662.25</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="160" ht="15.75" customHeight="1">
+    <row r="160" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B160" s="1">
-        <v>2549.57</v>
+        <v>-2549.5700000000002</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="161" ht="15.75" customHeight="1">
+    <row r="161" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B161" s="1">
-        <v>2843.19</v>
+        <v>-2843.19</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="162" ht="15.75" customHeight="1">
+    <row r="162" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>233</v>
       </c>
       <c r="B162" s="1">
-        <v>-835.65</v>
+        <v>835.65</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="163" ht="15.75" customHeight="1">
+    <row r="163" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>233</v>
       </c>
       <c r="B163" s="1">
-        <v>-93.73</v>
+        <v>93.73</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="164" ht="15.75" customHeight="1">
+    <row r="164" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>236</v>
       </c>
       <c r="B164" s="1">
-        <v>-386.79</v>
+        <v>386.79</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="165" ht="15.75" customHeight="1">
+    <row r="165" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>236</v>
       </c>
       <c r="B165" s="1">
-        <v>4250.11</v>
+        <v>-4250.1099999999997</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="166" ht="15.75" customHeight="1">
+    <row r="166" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>236</v>
       </c>
       <c r="B166" s="1">
-        <v>4316.14</v>
+        <v>-4316.1400000000003</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="167" ht="15.75" customHeight="1">
+    <row r="167" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
         <v>240</v>
       </c>
       <c r="B167" s="1">
-        <v>-1245.39</v>
+        <v>1245.3900000000001</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="168" ht="15.75" customHeight="1">
+    <row r="168" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
         <v>240</v>
       </c>
       <c r="B168" s="1">
-        <v>-1073.45</v>
+        <v>1073.45</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="169" ht="15.75" customHeight="1">
+    <row r="169" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
         <v>240</v>
       </c>
       <c r="B169" s="1">
-        <v>-364.13</v>
+        <v>364.13</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="170" ht="15.75" customHeight="1">
+    <row r="170" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
         <v>244</v>
       </c>
       <c r="B170" s="1">
-        <v>-1938.61</v>
+        <v>1938.61</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="171" ht="15.75" customHeight="1">
+    <row r="171" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
         <v>244</v>
       </c>
       <c r="B171" s="1">
-        <v>-1462.25</v>
+        <v>1462.25</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="172" ht="15.75" customHeight="1">
+    <row r="172" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
         <v>244</v>
       </c>
       <c r="B172" s="1">
-        <v>-792.87</v>
+        <v>792.87</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="173" ht="15.75" customHeight="1">
+    <row r="173" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
         <v>244</v>
       </c>
       <c r="B173" s="1">
-        <v>2926.55</v>
+        <v>-2926.55</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="174" ht="15.75" customHeight="1">
+    <row r="174" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
         <v>249</v>
       </c>
       <c r="B174" s="1">
-        <v>-809.54</v>
+        <v>809.54</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="175" ht="15.75" customHeight="1">
+    <row r="175" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="1" t="s">
         <v>249</v>
       </c>
       <c r="B175" s="1">
-        <v>-179.74</v>
+        <v>179.74</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="176" ht="15.75" customHeight="1">
+    <row r="176" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
         <v>249</v>
       </c>
       <c r="B176" s="1">
-        <v>-15.0</v>
+        <v>15</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="177" ht="15.75" customHeight="1">
+    <row r="177" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>249</v>
       </c>
       <c r="B177" s="1">
-        <v>9802.2</v>
+        <v>-9802.2000000000007</v>
       </c>
       <c r="C177" s="1" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="178" ht="15.75" customHeight="1">
+    <row r="178" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
         <v>254</v>
       </c>
       <c r="B178" s="1">
-        <v>-2400.64</v>
+        <v>2400.64</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="179" ht="15.75" customHeight="1">
+    <row r="179" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
         <v>254</v>
       </c>
       <c r="B179" s="1">
-        <v>-50.6</v>
+        <v>50.6</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="180" ht="15.75" customHeight="1">
+    <row r="180" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="1" t="s">
         <v>254</v>
       </c>
       <c r="B180" s="1">
-        <v>-49.78</v>
+        <v>49.78</v>
       </c>
       <c r="C180" s="1" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="181" ht="15.75" customHeight="1">
+    <row r="181" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="1" t="s">
         <v>258</v>
       </c>
       <c r="B181" s="1">
-        <v>-11322.43</v>
+        <v>11322.43</v>
       </c>
       <c r="C181" s="1" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="182" ht="15.75" customHeight="1">
+    <row r="182" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="1" t="s">
         <v>258</v>
       </c>
       <c r="B182" s="1">
-        <v>-6193.2</v>
+        <v>6193.2</v>
       </c>
       <c r="C182" s="1" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="183" ht="15.75" customHeight="1">
+    <row r="183" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="1" t="s">
         <v>258</v>
       </c>
       <c r="B183" s="1">
-        <v>-3361.51</v>
+        <v>3361.51</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="184" ht="15.75" customHeight="1">
+    <row r="184" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="1" t="s">
         <v>258</v>
       </c>
       <c r="B184" s="1">
-        <v>11302.82</v>
+        <v>-11302.82</v>
       </c>
       <c r="C184" s="1" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="185" ht="15.75" customHeight="1">
+    <row r="185" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="1" t="s">
         <v>263</v>
       </c>
       <c r="B185" s="1">
-        <v>-3012.01</v>
+        <v>3012.01</v>
       </c>
       <c r="C185" s="1" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="186" ht="15.75" customHeight="1">
+    <row r="186" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="1" t="s">
         <v>263</v>
       </c>
       <c r="B186" s="1">
-        <v>-1611.71</v>
+        <v>1611.71</v>
       </c>
       <c r="C186" s="1" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="187" ht="15.75" customHeight="1">
+    <row r="187" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="1" t="s">
         <v>263</v>
       </c>
       <c r="B187" s="1">
-        <v>1416.56</v>
+        <v>-1416.56</v>
       </c>
       <c r="C187" s="1" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="188" ht="15.75" customHeight="1">
+    <row r="188" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B188" s="1">
-        <v>-9172.9</v>
+        <v>9172.9</v>
       </c>
       <c r="C188" s="1" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="189" ht="15.75" customHeight="1">
+    <row r="189" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A189" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B189" s="1">
-        <v>-7574.8</v>
+        <v>7574.8</v>
       </c>
       <c r="C189" s="1" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="190" ht="15.75" customHeight="1">
+    <row r="190" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B190" s="1">
-        <v>-1678.99</v>
+        <v>1678.99</v>
       </c>
       <c r="C190" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="191" ht="15.75" customHeight="1">
+    <row r="191" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B191" s="1">
-        <v>-88.7</v>
+        <v>88.7</v>
       </c>
       <c r="C191" s="1" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="192" ht="15.75" customHeight="1">
+    <row r="192" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B192" s="1">
-        <v>407.69</v>
+        <v>-407.69</v>
       </c>
       <c r="C192" s="1" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="193" ht="15.75" customHeight="1">
+    <row r="193" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B193" s="1">
-        <v>2250.25</v>
+        <v>-2250.25</v>
       </c>
       <c r="C193" s="1" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="194" ht="15.75" customHeight="1">
+    <row r="194" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B194" s="1">
-        <v>3194.24</v>
+        <v>-3194.24</v>
       </c>
       <c r="C194" s="1" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="195" ht="15.75" customHeight="1">
+    <row r="195" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B195" s="1">
-        <v>6706.73</v>
+        <v>-6706.73</v>
       </c>
       <c r="C195" s="1" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="196" ht="15.75" customHeight="1">
+    <row r="196" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A196" s="1" t="s">
         <v>276</v>
       </c>
       <c r="B196" s="1">
-        <v>-801.8</v>
+        <v>801.8</v>
       </c>
       <c r="C196" s="1" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="197" ht="15.75" customHeight="1">
+    <row r="197" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A197" s="1" t="s">
         <v>278</v>
       </c>
       <c r="B197" s="1">
-        <v>-150.5</v>
+        <v>150.5</v>
       </c>
       <c r="C197" s="1" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="198" ht="15.75" customHeight="1">
+    <row r="198" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="1" t="s">
         <v>280</v>
       </c>
       <c r="B198" s="1">
-        <v>4245.33</v>
+        <v>-4245.33</v>
       </c>
       <c r="C198" s="1" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="199" ht="15.75" customHeight="1">
+    <row r="199" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="1" t="s">
         <v>282</v>
       </c>
       <c r="B199" s="1">
-        <v>6244.17</v>
+        <v>-6244.17</v>
       </c>
       <c r="C199" s="1" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="200" ht="15.75" customHeight="1">
+    <row r="200" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="1" t="s">
         <v>284</v>
       </c>
       <c r="B200" s="1">
-        <v>-751.39</v>
+        <v>751.39</v>
       </c>
       <c r="C200" s="1" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="201" ht="15.75" customHeight="1">
+    <row r="201" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="1" t="s">
         <v>286</v>
       </c>
       <c r="B201" s="1">
-        <v>-190.16</v>
+        <v>190.16</v>
       </c>
       <c r="C201" s="1" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="202" ht="15.75" customHeight="1"/>
-    <row r="203" ht="15.75" customHeight="1"/>
-    <row r="204" ht="15.75" customHeight="1"/>
-    <row r="205" ht="15.75" customHeight="1"/>
-    <row r="206" ht="15.75" customHeight="1"/>
-    <row r="207" ht="15.75" customHeight="1"/>
-    <row r="208" ht="15.75" customHeight="1"/>
-    <row r="209" ht="15.75" customHeight="1"/>
-    <row r="210" ht="15.75" customHeight="1"/>
-    <row r="211" ht="15.75" customHeight="1"/>
-    <row r="212" ht="15.75" customHeight="1"/>
-    <row r="213" ht="15.75" customHeight="1"/>
-    <row r="214" ht="15.75" customHeight="1"/>
-    <row r="215" ht="15.75" customHeight="1"/>
-    <row r="216" ht="15.75" customHeight="1"/>
-    <row r="217" ht="15.75" customHeight="1"/>
-    <row r="218" ht="15.75" customHeight="1"/>
-    <row r="219" ht="15.75" customHeight="1"/>
-    <row r="220" ht="15.75" customHeight="1"/>
-    <row r="221" ht="15.75" customHeight="1"/>
-    <row r="222" ht="15.75" customHeight="1"/>
-    <row r="223" ht="15.75" customHeight="1"/>
-    <row r="224" ht="15.75" customHeight="1"/>
-    <row r="225" ht="15.75" customHeight="1"/>
-    <row r="226" ht="15.75" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
-    <row r="228" ht="15.75" customHeight="1"/>
-    <row r="229" ht="15.75" customHeight="1"/>
-    <row r="230" ht="15.75" customHeight="1"/>
-    <row r="231" ht="15.75" customHeight="1"/>
-    <row r="232" ht="15.75" customHeight="1"/>
-    <row r="233" ht="15.75" customHeight="1"/>
-    <row r="234" ht="15.75" customHeight="1"/>
-    <row r="235" ht="15.75" customHeight="1"/>
-    <row r="236" ht="15.75" customHeight="1"/>
-    <row r="237" ht="15.75" customHeight="1"/>
-    <row r="238" ht="15.75" customHeight="1"/>
-    <row r="239" ht="15.75" customHeight="1"/>
-    <row r="240" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
-    <row r="249" ht="15.75" customHeight="1"/>
-    <row r="250" ht="15.75" customHeight="1"/>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
-    <row r="271" ht="15.75" customHeight="1"/>
-    <row r="272" ht="15.75" customHeight="1"/>
-    <row r="273" ht="15.75" customHeight="1"/>
-    <row r="274" ht="15.75" customHeight="1"/>
-    <row r="275" ht="15.75" customHeight="1"/>
-    <row r="276" ht="15.75" customHeight="1"/>
-    <row r="277" ht="15.75" customHeight="1"/>
-    <row r="278" ht="15.75" customHeight="1"/>
-    <row r="279" ht="15.75" customHeight="1"/>
-    <row r="280" ht="15.75" customHeight="1"/>
-    <row r="281" ht="15.75" customHeight="1"/>
-    <row r="282" ht="15.75" customHeight="1"/>
-    <row r="283" ht="15.75" customHeight="1"/>
-    <row r="284" ht="15.75" customHeight="1"/>
-    <row r="285" ht="15.75" customHeight="1"/>
-    <row r="286" ht="15.75" customHeight="1"/>
-    <row r="287" ht="15.75" customHeight="1"/>
-    <row r="288" ht="15.75" customHeight="1"/>
-    <row r="289" ht="15.75" customHeight="1"/>
-    <row r="290" ht="15.75" customHeight="1"/>
-    <row r="291" ht="15.75" customHeight="1"/>
-    <row r="292" ht="15.75" customHeight="1"/>
-    <row r="293" ht="15.75" customHeight="1"/>
-    <row r="294" ht="15.75" customHeight="1"/>
-    <row r="295" ht="15.75" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
-    <row r="298" ht="15.75" customHeight="1"/>
-    <row r="299" ht="15.75" customHeight="1"/>
-    <row r="300" ht="15.75" customHeight="1"/>
-    <row r="301" ht="15.75" customHeight="1"/>
-    <row r="302" ht="15.75" customHeight="1"/>
-    <row r="303" ht="15.75" customHeight="1"/>
-    <row r="304" ht="15.75" customHeight="1"/>
-    <row r="305" ht="15.75" customHeight="1"/>
-    <row r="306" ht="15.75" customHeight="1"/>
-    <row r="307" ht="15.75" customHeight="1"/>
-    <row r="308" ht="15.75" customHeight="1"/>
-    <row r="309" ht="15.75" customHeight="1"/>
-    <row r="310" ht="15.75" customHeight="1"/>
-    <row r="311" ht="15.75" customHeight="1"/>
-    <row r="312" ht="15.75" customHeight="1"/>
-    <row r="313" ht="15.75" customHeight="1"/>
-    <row r="314" ht="15.75" customHeight="1"/>
-    <row r="315" ht="15.75" customHeight="1"/>
-    <row r="316" ht="15.75" customHeight="1"/>
-    <row r="317" ht="15.75" customHeight="1"/>
-    <row r="318" ht="15.75" customHeight="1"/>
-    <row r="319" ht="15.75" customHeight="1"/>
-    <row r="320" ht="15.75" customHeight="1"/>
-    <row r="321" ht="15.75" customHeight="1"/>
-    <row r="322" ht="15.75" customHeight="1"/>
-    <row r="323" ht="15.75" customHeight="1"/>
-    <row r="324" ht="15.75" customHeight="1"/>
-    <row r="325" ht="15.75" customHeight="1"/>
-    <row r="326" ht="15.75" customHeight="1"/>
-    <row r="327" ht="15.75" customHeight="1"/>
-    <row r="328" ht="15.75" customHeight="1"/>
-    <row r="329" ht="15.75" customHeight="1"/>
-    <row r="330" ht="15.75" customHeight="1"/>
-    <row r="331" ht="15.75" customHeight="1"/>
-    <row r="332" ht="15.75" customHeight="1"/>
-    <row r="333" ht="15.75" customHeight="1"/>
-    <row r="334" ht="15.75" customHeight="1"/>
-    <row r="335" ht="15.75" customHeight="1"/>
-    <row r="336" ht="15.75" customHeight="1"/>
-    <row r="337" ht="15.75" customHeight="1"/>
-    <row r="338" ht="15.75" customHeight="1"/>
-    <row r="339" ht="15.75" customHeight="1"/>
-    <row r="340" ht="15.75" customHeight="1"/>
-    <row r="341" ht="15.75" customHeight="1"/>
-    <row r="342" ht="15.75" customHeight="1"/>
-    <row r="343" ht="15.75" customHeight="1"/>
-    <row r="344" ht="15.75" customHeight="1"/>
-    <row r="345" ht="15.75" customHeight="1"/>
-    <row r="346" ht="15.75" customHeight="1"/>
-    <row r="347" ht="15.75" customHeight="1"/>
-    <row r="348" ht="15.75" customHeight="1"/>
-    <row r="349" ht="15.75" customHeight="1"/>
-    <row r="350" ht="15.75" customHeight="1"/>
-    <row r="351" ht="15.75" customHeight="1"/>
-    <row r="352" ht="15.75" customHeight="1"/>
-    <row r="353" ht="15.75" customHeight="1"/>
-    <row r="354" ht="15.75" customHeight="1"/>
-    <row r="355" ht="15.75" customHeight="1"/>
-    <row r="356" ht="15.75" customHeight="1"/>
-    <row r="357" ht="15.75" customHeight="1"/>
-    <row r="358" ht="15.75" customHeight="1"/>
-    <row r="359" ht="15.75" customHeight="1"/>
-    <row r="360" ht="15.75" customHeight="1"/>
-    <row r="361" ht="15.75" customHeight="1"/>
-    <row r="362" ht="15.75" customHeight="1"/>
-    <row r="363" ht="15.75" customHeight="1"/>
-    <row r="364" ht="15.75" customHeight="1"/>
-    <row r="365" ht="15.75" customHeight="1"/>
-    <row r="366" ht="15.75" customHeight="1"/>
-    <row r="367" ht="15.75" customHeight="1"/>
-    <row r="368" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
-    <row r="385" ht="15.75" customHeight="1"/>
-    <row r="386" ht="15.75" customHeight="1"/>
-    <row r="387" ht="15.75" customHeight="1"/>
-    <row r="388" ht="15.75" customHeight="1"/>
-    <row r="389" ht="15.75" customHeight="1"/>
-    <row r="390" ht="15.75" customHeight="1"/>
-    <row r="391" ht="15.75" customHeight="1"/>
-    <row r="392" ht="15.75" customHeight="1"/>
-    <row r="393" ht="15.75" customHeight="1"/>
-    <row r="394" ht="15.75" customHeight="1"/>
-    <row r="395" ht="15.75" customHeight="1"/>
-    <row r="396" ht="15.75" customHeight="1"/>
-    <row r="397" ht="15.75" customHeight="1"/>
-    <row r="398" ht="15.75" customHeight="1"/>
-    <row r="399" ht="15.75" customHeight="1"/>
-    <row r="400" ht="15.75" customHeight="1"/>
-    <row r="401" ht="15.75" customHeight="1"/>
-    <row r="402" ht="15.75" customHeight="1"/>
-    <row r="403" ht="15.75" customHeight="1"/>
-    <row r="404" ht="15.75" customHeight="1"/>
-    <row r="405" ht="15.75" customHeight="1"/>
-    <row r="406" ht="15.75" customHeight="1"/>
-    <row r="407" ht="15.75" customHeight="1"/>
-    <row r="408" ht="15.75" customHeight="1"/>
-    <row r="409" ht="15.75" customHeight="1"/>
-    <row r="410" ht="15.75" customHeight="1"/>
-    <row r="411" ht="15.75" customHeight="1"/>
-    <row r="412" ht="15.75" customHeight="1"/>
-    <row r="413" ht="15.75" customHeight="1"/>
-    <row r="414" ht="15.75" customHeight="1"/>
-    <row r="415" ht="15.75" customHeight="1"/>
-    <row r="416" ht="15.75" customHeight="1"/>
-    <row r="417" ht="15.75" customHeight="1"/>
-    <row r="418" ht="15.75" customHeight="1"/>
-    <row r="419" ht="15.75" customHeight="1"/>
-    <row r="420" ht="15.75" customHeight="1"/>
-    <row r="421" ht="15.75" customHeight="1"/>
-    <row r="422" ht="15.75" customHeight="1"/>
-    <row r="423" ht="15.75" customHeight="1"/>
-    <row r="424" ht="15.75" customHeight="1"/>
-    <row r="425" ht="15.75" customHeight="1"/>
-    <row r="426" ht="15.75" customHeight="1"/>
-    <row r="427" ht="15.75" customHeight="1"/>
-    <row r="428" ht="15.75" customHeight="1"/>
-    <row r="429" ht="15.75" customHeight="1"/>
-    <row r="430" ht="15.75" customHeight="1"/>
-    <row r="431" ht="15.75" customHeight="1"/>
-    <row r="432" ht="15.75" customHeight="1"/>
-    <row r="433" ht="15.75" customHeight="1"/>
-    <row r="434" ht="15.75" customHeight="1"/>
-    <row r="435" ht="15.75" customHeight="1"/>
-    <row r="436" ht="15.75" customHeight="1"/>
-    <row r="437" ht="15.75" customHeight="1"/>
-    <row r="438" ht="15.75" customHeight="1"/>
-    <row r="439" ht="15.75" customHeight="1"/>
-    <row r="440" ht="15.75" customHeight="1"/>
-    <row r="441" ht="15.75" customHeight="1"/>
-    <row r="442" ht="15.75" customHeight="1"/>
-    <row r="443" ht="15.75" customHeight="1"/>
-    <row r="444" ht="15.75" customHeight="1"/>
-    <row r="445" ht="15.75" customHeight="1"/>
-    <row r="446" ht="15.75" customHeight="1"/>
-    <row r="447" ht="15.75" customHeight="1"/>
-    <row r="448" ht="15.75" customHeight="1"/>
-    <row r="449" ht="15.75" customHeight="1"/>
-    <row r="450" ht="15.75" customHeight="1"/>
-    <row r="451" ht="15.75" customHeight="1"/>
-    <row r="452" ht="15.75" customHeight="1"/>
-    <row r="453" ht="15.75" customHeight="1"/>
-    <row r="454" ht="15.75" customHeight="1"/>
-    <row r="455" ht="15.75" customHeight="1"/>
-    <row r="456" ht="15.75" customHeight="1"/>
-    <row r="457" ht="15.75" customHeight="1"/>
-    <row r="458" ht="15.75" customHeight="1"/>
-    <row r="459" ht="15.75" customHeight="1"/>
-    <row r="460" ht="15.75" customHeight="1"/>
-    <row r="461" ht="15.75" customHeight="1"/>
-    <row r="462" ht="15.75" customHeight="1"/>
-    <row r="463" ht="15.75" customHeight="1"/>
-    <row r="464" ht="15.75" customHeight="1"/>
-    <row r="465" ht="15.75" customHeight="1"/>
-    <row r="466" ht="15.75" customHeight="1"/>
-    <row r="467" ht="15.75" customHeight="1"/>
-    <row r="468" ht="15.75" customHeight="1"/>
-    <row r="469" ht="15.75" customHeight="1"/>
-    <row r="470" ht="15.75" customHeight="1"/>
-    <row r="471" ht="15.75" customHeight="1"/>
-    <row r="472" ht="15.75" customHeight="1"/>
-    <row r="473" ht="15.75" customHeight="1"/>
-    <row r="474" ht="15.75" customHeight="1"/>
-    <row r="475" ht="15.75" customHeight="1"/>
-    <row r="476" ht="15.75" customHeight="1"/>
-    <row r="477" ht="15.75" customHeight="1"/>
-    <row r="478" ht="15.75" customHeight="1"/>
-    <row r="479" ht="15.75" customHeight="1"/>
-    <row r="480" ht="15.75" customHeight="1"/>
-    <row r="481" ht="15.75" customHeight="1"/>
-    <row r="482" ht="15.75" customHeight="1"/>
-    <row r="483" ht="15.75" customHeight="1"/>
-    <row r="484" ht="15.75" customHeight="1"/>
-    <row r="485" ht="15.75" customHeight="1"/>
-    <row r="486" ht="15.75" customHeight="1"/>
-    <row r="487" ht="15.75" customHeight="1"/>
-    <row r="488" ht="15.75" customHeight="1"/>
-    <row r="489" ht="15.75" customHeight="1"/>
-    <row r="490" ht="15.75" customHeight="1"/>
-    <row r="491" ht="15.75" customHeight="1"/>
-    <row r="492" ht="15.75" customHeight="1"/>
-    <row r="493" ht="15.75" customHeight="1"/>
-    <row r="494" ht="15.75" customHeight="1"/>
-    <row r="495" ht="15.75" customHeight="1"/>
-    <row r="496" ht="15.75" customHeight="1"/>
-    <row r="497" ht="15.75" customHeight="1"/>
-    <row r="498" ht="15.75" customHeight="1"/>
-    <row r="499" ht="15.75" customHeight="1"/>
-    <row r="500" ht="15.75" customHeight="1"/>
-    <row r="501" ht="15.75" customHeight="1"/>
-    <row r="502" ht="15.75" customHeight="1"/>
-    <row r="503" ht="15.75" customHeight="1"/>
-    <row r="504" ht="15.75" customHeight="1"/>
-    <row r="505" ht="15.75" customHeight="1"/>
-    <row r="506" ht="15.75" customHeight="1"/>
-    <row r="507" ht="15.75" customHeight="1"/>
-    <row r="508" ht="15.75" customHeight="1"/>
-    <row r="509" ht="15.75" customHeight="1"/>
-    <row r="510" ht="15.75" customHeight="1"/>
-    <row r="511" ht="15.75" customHeight="1"/>
-    <row r="512" ht="15.75" customHeight="1"/>
-    <row r="513" ht="15.75" customHeight="1"/>
-    <row r="514" ht="15.75" customHeight="1"/>
-    <row r="515" ht="15.75" customHeight="1"/>
-    <row r="516" ht="15.75" customHeight="1"/>
-    <row r="517" ht="15.75" customHeight="1"/>
-    <row r="518" ht="15.75" customHeight="1"/>
-    <row r="519" ht="15.75" customHeight="1"/>
-    <row r="520" ht="15.75" customHeight="1"/>
-    <row r="521" ht="15.75" customHeight="1"/>
-    <row r="522" ht="15.75" customHeight="1"/>
-    <row r="523" ht="15.75" customHeight="1"/>
-    <row r="524" ht="15.75" customHeight="1"/>
-    <row r="525" ht="15.75" customHeight="1"/>
-    <row r="526" ht="15.75" customHeight="1"/>
-    <row r="527" ht="15.75" customHeight="1"/>
-    <row r="528" ht="15.75" customHeight="1"/>
-    <row r="529" ht="15.75" customHeight="1"/>
-    <row r="530" ht="15.75" customHeight="1"/>
-    <row r="531" ht="15.75" customHeight="1"/>
-    <row r="532" ht="15.75" customHeight="1"/>
-    <row r="533" ht="15.75" customHeight="1"/>
-    <row r="534" ht="15.75" customHeight="1"/>
-    <row r="535" ht="15.75" customHeight="1"/>
-    <row r="536" ht="15.75" customHeight="1"/>
-    <row r="537" ht="15.75" customHeight="1"/>
-    <row r="538" ht="15.75" customHeight="1"/>
-    <row r="539" ht="15.75" customHeight="1"/>
-    <row r="540" ht="15.75" customHeight="1"/>
-    <row r="541" ht="15.75" customHeight="1"/>
-    <row r="542" ht="15.75" customHeight="1"/>
-    <row r="543" ht="15.75" customHeight="1"/>
-    <row r="544" ht="15.75" customHeight="1"/>
-    <row r="545" ht="15.75" customHeight="1"/>
-    <row r="546" ht="15.75" customHeight="1"/>
-    <row r="547" ht="15.75" customHeight="1"/>
-    <row r="548" ht="15.75" customHeight="1"/>
-    <row r="549" ht="15.75" customHeight="1"/>
-    <row r="550" ht="15.75" customHeight="1"/>
-    <row r="551" ht="15.75" customHeight="1"/>
-    <row r="552" ht="15.75" customHeight="1"/>
-    <row r="553" ht="15.75" customHeight="1"/>
-    <row r="554" ht="15.75" customHeight="1"/>
-    <row r="555" ht="15.75" customHeight="1"/>
-    <row r="556" ht="15.75" customHeight="1"/>
-    <row r="557" ht="15.75" customHeight="1"/>
-    <row r="558" ht="15.75" customHeight="1"/>
-    <row r="559" ht="15.75" customHeight="1"/>
-    <row r="560" ht="15.75" customHeight="1"/>
-    <row r="561" ht="15.75" customHeight="1"/>
-    <row r="562" ht="15.75" customHeight="1"/>
-    <row r="563" ht="15.75" customHeight="1"/>
-    <row r="564" ht="15.75" customHeight="1"/>
-    <row r="565" ht="15.75" customHeight="1"/>
-    <row r="566" ht="15.75" customHeight="1"/>
-    <row r="567" ht="15.75" customHeight="1"/>
-    <row r="568" ht="15.75" customHeight="1"/>
-    <row r="569" ht="15.75" customHeight="1"/>
-    <row r="570" ht="15.75" customHeight="1"/>
-    <row r="571" ht="15.75" customHeight="1"/>
-    <row r="572" ht="15.75" customHeight="1"/>
-    <row r="573" ht="15.75" customHeight="1"/>
-    <row r="574" ht="15.75" customHeight="1"/>
-    <row r="575" ht="15.75" customHeight="1"/>
-    <row r="576" ht="15.75" customHeight="1"/>
-    <row r="577" ht="15.75" customHeight="1"/>
-    <row r="578" ht="15.75" customHeight="1"/>
-    <row r="579" ht="15.75" customHeight="1"/>
-    <row r="580" ht="15.75" customHeight="1"/>
-    <row r="581" ht="15.75" customHeight="1"/>
-    <row r="582" ht="15.75" customHeight="1"/>
-    <row r="583" ht="15.75" customHeight="1"/>
-    <row r="584" ht="15.75" customHeight="1"/>
-    <row r="585" ht="15.75" customHeight="1"/>
-    <row r="586" ht="15.75" customHeight="1"/>
-    <row r="587" ht="15.75" customHeight="1"/>
-    <row r="588" ht="15.75" customHeight="1"/>
-    <row r="589" ht="15.75" customHeight="1"/>
-    <row r="590" ht="15.75" customHeight="1"/>
-    <row r="591" ht="15.75" customHeight="1"/>
-    <row r="592" ht="15.75" customHeight="1"/>
-    <row r="593" ht="15.75" customHeight="1"/>
-    <row r="594" ht="15.75" customHeight="1"/>
-    <row r="595" ht="15.75" customHeight="1"/>
-    <row r="596" ht="15.75" customHeight="1"/>
-    <row r="597" ht="15.75" customHeight="1"/>
-    <row r="598" ht="15.75" customHeight="1"/>
-    <row r="599" ht="15.75" customHeight="1"/>
-    <row r="600" ht="15.75" customHeight="1"/>
-    <row r="601" ht="15.75" customHeight="1"/>
-    <row r="602" ht="15.75" customHeight="1"/>
-    <row r="603" ht="15.75" customHeight="1"/>
-    <row r="604" ht="15.75" customHeight="1"/>
-    <row r="605" ht="15.75" customHeight="1"/>
-    <row r="606" ht="15.75" customHeight="1"/>
-    <row r="607" ht="15.75" customHeight="1"/>
-    <row r="608" ht="15.75" customHeight="1"/>
-    <row r="609" ht="15.75" customHeight="1"/>
-    <row r="610" ht="15.75" customHeight="1"/>
-    <row r="611" ht="15.75" customHeight="1"/>
-    <row r="612" ht="15.75" customHeight="1"/>
-    <row r="613" ht="15.75" customHeight="1"/>
-    <row r="614" ht="15.75" customHeight="1"/>
-    <row r="615" ht="15.75" customHeight="1"/>
-    <row r="616" ht="15.75" customHeight="1"/>
-    <row r="617" ht="15.75" customHeight="1"/>
-    <row r="618" ht="15.75" customHeight="1"/>
-    <row r="619" ht="15.75" customHeight="1"/>
-    <row r="620" ht="15.75" customHeight="1"/>
-    <row r="621" ht="15.75" customHeight="1"/>
-    <row r="622" ht="15.75" customHeight="1"/>
-    <row r="623" ht="15.75" customHeight="1"/>
-    <row r="624" ht="15.75" customHeight="1"/>
-    <row r="625" ht="15.75" customHeight="1"/>
-    <row r="626" ht="15.75" customHeight="1"/>
-    <row r="627" ht="15.75" customHeight="1"/>
-    <row r="628" ht="15.75" customHeight="1"/>
-    <row r="629" ht="15.75" customHeight="1"/>
-    <row r="630" ht="15.75" customHeight="1"/>
-    <row r="631" ht="15.75" customHeight="1"/>
-    <row r="632" ht="15.75" customHeight="1"/>
-    <row r="633" ht="15.75" customHeight="1"/>
-    <row r="634" ht="15.75" customHeight="1"/>
-    <row r="635" ht="15.75" customHeight="1"/>
-    <row r="636" ht="15.75" customHeight="1"/>
-    <row r="637" ht="15.75" customHeight="1"/>
-    <row r="638" ht="15.75" customHeight="1"/>
-    <row r="639" ht="15.75" customHeight="1"/>
-    <row r="640" ht="15.75" customHeight="1"/>
-    <row r="641" ht="15.75" customHeight="1"/>
-    <row r="642" ht="15.75" customHeight="1"/>
-    <row r="643" ht="15.75" customHeight="1"/>
-    <row r="644" ht="15.75" customHeight="1"/>
-    <row r="645" ht="15.75" customHeight="1"/>
-    <row r="646" ht="15.75" customHeight="1"/>
-    <row r="647" ht="15.75" customHeight="1"/>
-    <row r="648" ht="15.75" customHeight="1"/>
-    <row r="649" ht="15.75" customHeight="1"/>
-    <row r="650" ht="15.75" customHeight="1"/>
-    <row r="651" ht="15.75" customHeight="1"/>
-    <row r="652" ht="15.75" customHeight="1"/>
-    <row r="653" ht="15.75" customHeight="1"/>
-    <row r="654" ht="15.75" customHeight="1"/>
-    <row r="655" ht="15.75" customHeight="1"/>
-    <row r="656" ht="15.75" customHeight="1"/>
-    <row r="657" ht="15.75" customHeight="1"/>
-    <row r="658" ht="15.75" customHeight="1"/>
-    <row r="659" ht="15.75" customHeight="1"/>
-    <row r="660" ht="15.75" customHeight="1"/>
-    <row r="661" ht="15.75" customHeight="1"/>
-    <row r="662" ht="15.75" customHeight="1"/>
-    <row r="663" ht="15.75" customHeight="1"/>
-    <row r="664" ht="15.75" customHeight="1"/>
-    <row r="665" ht="15.75" customHeight="1"/>
-    <row r="666" ht="15.75" customHeight="1"/>
-    <row r="667" ht="15.75" customHeight="1"/>
-    <row r="668" ht="15.75" customHeight="1"/>
-    <row r="669" ht="15.75" customHeight="1"/>
-    <row r="670" ht="15.75" customHeight="1"/>
-    <row r="671" ht="15.75" customHeight="1"/>
-    <row r="672" ht="15.75" customHeight="1"/>
-    <row r="673" ht="15.75" customHeight="1"/>
-    <row r="674" ht="15.75" customHeight="1"/>
-    <row r="675" ht="15.75" customHeight="1"/>
-    <row r="676" ht="15.75" customHeight="1"/>
-    <row r="677" ht="15.75" customHeight="1"/>
-    <row r="678" ht="15.75" customHeight="1"/>
-    <row r="679" ht="15.75" customHeight="1"/>
-    <row r="680" ht="15.75" customHeight="1"/>
-    <row r="681" ht="15.75" customHeight="1"/>
-    <row r="682" ht="15.75" customHeight="1"/>
-    <row r="683" ht="15.75" customHeight="1"/>
-    <row r="684" ht="15.75" customHeight="1"/>
-    <row r="685" ht="15.75" customHeight="1"/>
-    <row r="686" ht="15.75" customHeight="1"/>
-    <row r="687" ht="15.75" customHeight="1"/>
-    <row r="688" ht="15.75" customHeight="1"/>
-    <row r="689" ht="15.75" customHeight="1"/>
-    <row r="690" ht="15.75" customHeight="1"/>
-    <row r="691" ht="15.75" customHeight="1"/>
-    <row r="692" ht="15.75" customHeight="1"/>
-    <row r="693" ht="15.75" customHeight="1"/>
-    <row r="694" ht="15.75" customHeight="1"/>
-    <row r="695" ht="15.75" customHeight="1"/>
-    <row r="696" ht="15.75" customHeight="1"/>
-    <row r="697" ht="15.75" customHeight="1"/>
-    <row r="698" ht="15.75" customHeight="1"/>
-    <row r="699" ht="15.75" customHeight="1"/>
-    <row r="700" ht="15.75" customHeight="1"/>
-    <row r="701" ht="15.75" customHeight="1"/>
-    <row r="702" ht="15.75" customHeight="1"/>
-    <row r="703" ht="15.75" customHeight="1"/>
-    <row r="704" ht="15.75" customHeight="1"/>
-    <row r="705" ht="15.75" customHeight="1"/>
-    <row r="706" ht="15.75" customHeight="1"/>
-    <row r="707" ht="15.75" customHeight="1"/>
-    <row r="708" ht="15.75" customHeight="1"/>
-    <row r="709" ht="15.75" customHeight="1"/>
-    <row r="710" ht="15.75" customHeight="1"/>
-    <row r="711" ht="15.75" customHeight="1"/>
-    <row r="712" ht="15.75" customHeight="1"/>
-    <row r="713" ht="15.75" customHeight="1"/>
-    <row r="714" ht="15.75" customHeight="1"/>
-    <row r="715" ht="15.75" customHeight="1"/>
-    <row r="716" ht="15.75" customHeight="1"/>
-    <row r="717" ht="15.75" customHeight="1"/>
-    <row r="718" ht="15.75" customHeight="1"/>
-    <row r="719" ht="15.75" customHeight="1"/>
-    <row r="720" ht="15.75" customHeight="1"/>
-    <row r="721" ht="15.75" customHeight="1"/>
-    <row r="722" ht="15.75" customHeight="1"/>
-    <row r="723" ht="15.75" customHeight="1"/>
-    <row r="724" ht="15.75" customHeight="1"/>
-    <row r="725" ht="15.75" customHeight="1"/>
-    <row r="726" ht="15.75" customHeight="1"/>
-    <row r="727" ht="15.75" customHeight="1"/>
-    <row r="728" ht="15.75" customHeight="1"/>
-    <row r="729" ht="15.75" customHeight="1"/>
-    <row r="730" ht="15.75" customHeight="1"/>
-    <row r="731" ht="15.75" customHeight="1"/>
-    <row r="732" ht="15.75" customHeight="1"/>
-    <row r="733" ht="15.75" customHeight="1"/>
-    <row r="734" ht="15.75" customHeight="1"/>
-    <row r="735" ht="15.75" customHeight="1"/>
-    <row r="736" ht="15.75" customHeight="1"/>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
-    <row r="750" ht="15.75" customHeight="1"/>
-    <row r="751" ht="15.75" customHeight="1"/>
-    <row r="752" ht="15.75" customHeight="1"/>
-    <row r="753" ht="15.75" customHeight="1"/>
-    <row r="754" ht="15.75" customHeight="1"/>
-    <row r="755" ht="15.75" customHeight="1"/>
-    <row r="756" ht="15.75" customHeight="1"/>
-    <row r="757" ht="15.75" customHeight="1"/>
-    <row r="758" ht="15.75" customHeight="1"/>
-    <row r="759" ht="15.75" customHeight="1"/>
-    <row r="760" ht="15.75" customHeight="1"/>
-    <row r="761" ht="15.75" customHeight="1"/>
-    <row r="762" ht="15.75" customHeight="1"/>
-    <row r="763" ht="15.75" customHeight="1"/>
-    <row r="764" ht="15.75" customHeight="1"/>
-    <row r="765" ht="15.75" customHeight="1"/>
-    <row r="766" ht="15.75" customHeight="1"/>
-    <row r="767" ht="15.75" customHeight="1"/>
-    <row r="768" ht="15.75" customHeight="1"/>
-    <row r="769" ht="15.75" customHeight="1"/>
-    <row r="770" ht="15.75" customHeight="1"/>
-    <row r="771" ht="15.75" customHeight="1"/>
-    <row r="772" ht="15.75" customHeight="1"/>
-    <row r="773" ht="15.75" customHeight="1"/>
-    <row r="774" ht="15.75" customHeight="1"/>
-    <row r="775" ht="15.75" customHeight="1"/>
-    <row r="776" ht="15.75" customHeight="1"/>
-    <row r="777" ht="15.75" customHeight="1"/>
-    <row r="778" ht="15.75" customHeight="1"/>
-    <row r="779" ht="15.75" customHeight="1"/>
-    <row r="780" ht="15.75" customHeight="1"/>
-    <row r="781" ht="15.75" customHeight="1"/>
-    <row r="782" ht="15.75" customHeight="1"/>
-    <row r="783" ht="15.75" customHeight="1"/>
-    <row r="784" ht="15.75" customHeight="1"/>
-    <row r="785" ht="15.75" customHeight="1"/>
-    <row r="786" ht="15.75" customHeight="1"/>
-    <row r="787" ht="15.75" customHeight="1"/>
-    <row r="788" ht="15.75" customHeight="1"/>
-    <row r="789" ht="15.75" customHeight="1"/>
-    <row r="790" ht="15.75" customHeight="1"/>
-    <row r="791" ht="15.75" customHeight="1"/>
-    <row r="792" ht="15.75" customHeight="1"/>
-    <row r="793" ht="15.75" customHeight="1"/>
-    <row r="794" ht="15.75" customHeight="1"/>
-    <row r="795" ht="15.75" customHeight="1"/>
-    <row r="796" ht="15.75" customHeight="1"/>
-    <row r="797" ht="15.75" customHeight="1"/>
-    <row r="798" ht="15.75" customHeight="1"/>
-    <row r="799" ht="15.75" customHeight="1"/>
-    <row r="800" ht="15.75" customHeight="1"/>
-    <row r="801" ht="15.75" customHeight="1"/>
-    <row r="802" ht="15.75" customHeight="1"/>
-    <row r="803" ht="15.75" customHeight="1"/>
-    <row r="804" ht="15.75" customHeight="1"/>
-    <row r="805" ht="15.75" customHeight="1"/>
-    <row r="806" ht="15.75" customHeight="1"/>
-    <row r="807" ht="15.75" customHeight="1"/>
-    <row r="808" ht="15.75" customHeight="1"/>
-    <row r="809" ht="15.75" customHeight="1"/>
-    <row r="810" ht="15.75" customHeight="1"/>
-    <row r="811" ht="15.75" customHeight="1"/>
-    <row r="812" ht="15.75" customHeight="1"/>
-    <row r="813" ht="15.75" customHeight="1"/>
-    <row r="814" ht="15.75" customHeight="1"/>
-    <row r="815" ht="15.75" customHeight="1"/>
-    <row r="816" ht="15.75" customHeight="1"/>
-    <row r="817" ht="15.75" customHeight="1"/>
-    <row r="818" ht="15.75" customHeight="1"/>
-    <row r="819" ht="15.75" customHeight="1"/>
-    <row r="820" ht="15.75" customHeight="1"/>
-    <row r="821" ht="15.75" customHeight="1"/>
-    <row r="822" ht="15.75" customHeight="1"/>
-    <row r="823" ht="15.75" customHeight="1"/>
-    <row r="824" ht="15.75" customHeight="1"/>
-    <row r="825" ht="15.75" customHeight="1"/>
-    <row r="826" ht="15.75" customHeight="1"/>
-    <row r="827" ht="15.75" customHeight="1"/>
-    <row r="828" ht="15.75" customHeight="1"/>
-    <row r="829" ht="15.75" customHeight="1"/>
-    <row r="830" ht="15.75" customHeight="1"/>
-    <row r="831" ht="15.75" customHeight="1"/>
-    <row r="832" ht="15.75" customHeight="1"/>
-    <row r="833" ht="15.75" customHeight="1"/>
-    <row r="834" ht="15.75" customHeight="1"/>
-    <row r="835" ht="15.75" customHeight="1"/>
-    <row r="836" ht="15.75" customHeight="1"/>
-    <row r="837" ht="15.75" customHeight="1"/>
-    <row r="838" ht="15.75" customHeight="1"/>
-    <row r="839" ht="15.75" customHeight="1"/>
-    <row r="840" ht="15.75" customHeight="1"/>
-    <row r="841" ht="15.75" customHeight="1"/>
-    <row r="842" ht="15.75" customHeight="1"/>
-    <row r="843" ht="15.75" customHeight="1"/>
-    <row r="844" ht="15.75" customHeight="1"/>
-    <row r="845" ht="15.75" customHeight="1"/>
-    <row r="846" ht="15.75" customHeight="1"/>
-    <row r="847" ht="15.75" customHeight="1"/>
-    <row r="848" ht="15.75" customHeight="1"/>
-    <row r="849" ht="15.75" customHeight="1"/>
-    <row r="850" ht="15.75" customHeight="1"/>
-    <row r="851" ht="15.75" customHeight="1"/>
-    <row r="852" ht="15.75" customHeight="1"/>
-    <row r="853" ht="15.75" customHeight="1"/>
-    <row r="854" ht="15.75" customHeight="1"/>
-    <row r="855" ht="15.75" customHeight="1"/>
-    <row r="856" ht="15.75" customHeight="1"/>
-    <row r="857" ht="15.75" customHeight="1"/>
-    <row r="858" ht="15.75" customHeight="1"/>
-    <row r="859" ht="15.75" customHeight="1"/>
-    <row r="860" ht="15.75" customHeight="1"/>
-    <row r="861" ht="15.75" customHeight="1"/>
-    <row r="862" ht="15.75" customHeight="1"/>
-    <row r="863" ht="15.75" customHeight="1"/>
-    <row r="864" ht="15.75" customHeight="1"/>
-    <row r="865" ht="15.75" customHeight="1"/>
-    <row r="866" ht="15.75" customHeight="1"/>
-    <row r="867" ht="15.75" customHeight="1"/>
-    <row r="868" ht="15.75" customHeight="1"/>
-    <row r="869" ht="15.75" customHeight="1"/>
-    <row r="870" ht="15.75" customHeight="1"/>
-    <row r="871" ht="15.75" customHeight="1"/>
-    <row r="872" ht="15.75" customHeight="1"/>
-    <row r="873" ht="15.75" customHeight="1"/>
-    <row r="874" ht="15.75" customHeight="1"/>
-    <row r="875" ht="15.75" customHeight="1"/>
-    <row r="876" ht="15.75" customHeight="1"/>
-    <row r="877" ht="15.75" customHeight="1"/>
-    <row r="878" ht="15.75" customHeight="1"/>
-    <row r="879" ht="15.75" customHeight="1"/>
-    <row r="880" ht="15.75" customHeight="1"/>
-    <row r="881" ht="15.75" customHeight="1"/>
-    <row r="882" ht="15.75" customHeight="1"/>
-    <row r="883" ht="15.75" customHeight="1"/>
-    <row r="884" ht="15.75" customHeight="1"/>
-    <row r="885" ht="15.75" customHeight="1"/>
-    <row r="886" ht="15.75" customHeight="1"/>
-    <row r="887" ht="15.75" customHeight="1"/>
-    <row r="888" ht="15.75" customHeight="1"/>
-    <row r="889" ht="15.75" customHeight="1"/>
-    <row r="890" ht="15.75" customHeight="1"/>
-    <row r="891" ht="15.75" customHeight="1"/>
-    <row r="892" ht="15.75" customHeight="1"/>
-    <row r="893" ht="15.75" customHeight="1"/>
-    <row r="894" ht="15.75" customHeight="1"/>
-    <row r="895" ht="15.75" customHeight="1"/>
-    <row r="896" ht="15.75" customHeight="1"/>
-    <row r="897" ht="15.75" customHeight="1"/>
-    <row r="898" ht="15.75" customHeight="1"/>
-    <row r="899" ht="15.75" customHeight="1"/>
-    <row r="900" ht="15.75" customHeight="1"/>
-    <row r="901" ht="15.75" customHeight="1"/>
-    <row r="902" ht="15.75" customHeight="1"/>
-    <row r="903" ht="15.75" customHeight="1"/>
-    <row r="904" ht="15.75" customHeight="1"/>
-    <row r="905" ht="15.75" customHeight="1"/>
-    <row r="906" ht="15.75" customHeight="1"/>
-    <row r="907" ht="15.75" customHeight="1"/>
-    <row r="908" ht="15.75" customHeight="1"/>
-    <row r="909" ht="15.75" customHeight="1"/>
-    <row r="910" ht="15.75" customHeight="1"/>
-    <row r="911" ht="15.75" customHeight="1"/>
-    <row r="912" ht="15.75" customHeight="1"/>
-    <row r="913" ht="15.75" customHeight="1"/>
-    <row r="914" ht="15.75" customHeight="1"/>
-    <row r="915" ht="15.75" customHeight="1"/>
-    <row r="916" ht="15.75" customHeight="1"/>
-    <row r="917" ht="15.75" customHeight="1"/>
-    <row r="918" ht="15.75" customHeight="1"/>
-    <row r="919" ht="15.75" customHeight="1"/>
-    <row r="920" ht="15.75" customHeight="1"/>
-    <row r="921" ht="15.75" customHeight="1"/>
-    <row r="922" ht="15.75" customHeight="1"/>
-    <row r="923" ht="15.75" customHeight="1"/>
-    <row r="924" ht="15.75" customHeight="1"/>
-    <row r="925" ht="15.75" customHeight="1"/>
-    <row r="926" ht="15.75" customHeight="1"/>
-    <row r="927" ht="15.75" customHeight="1"/>
-    <row r="928" ht="15.75" customHeight="1"/>
-    <row r="929" ht="15.75" customHeight="1"/>
-    <row r="930" ht="15.75" customHeight="1"/>
-    <row r="931" ht="15.75" customHeight="1"/>
-    <row r="932" ht="15.75" customHeight="1"/>
-    <row r="933" ht="15.75" customHeight="1"/>
-    <row r="934" ht="15.75" customHeight="1"/>
-    <row r="935" ht="15.75" customHeight="1"/>
-    <row r="936" ht="15.75" customHeight="1"/>
-    <row r="937" ht="15.75" customHeight="1"/>
-    <row r="938" ht="15.75" customHeight="1"/>
-    <row r="939" ht="15.75" customHeight="1"/>
-    <row r="940" ht="15.75" customHeight="1"/>
-    <row r="941" ht="15.75" customHeight="1"/>
-    <row r="942" ht="15.75" customHeight="1"/>
-    <row r="943" ht="15.75" customHeight="1"/>
-    <row r="944" ht="15.75" customHeight="1"/>
-    <row r="945" ht="15.75" customHeight="1"/>
-    <row r="946" ht="15.75" customHeight="1"/>
-    <row r="947" ht="15.75" customHeight="1"/>
-    <row r="948" ht="15.75" customHeight="1"/>
-    <row r="949" ht="15.75" customHeight="1"/>
-    <row r="950" ht="15.75" customHeight="1"/>
-    <row r="951" ht="15.75" customHeight="1"/>
-    <row r="952" ht="15.75" customHeight="1"/>
-    <row r="953" ht="15.75" customHeight="1"/>
-    <row r="954" ht="15.75" customHeight="1"/>
-    <row r="955" ht="15.75" customHeight="1"/>
-    <row r="956" ht="15.75" customHeight="1"/>
-    <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="202" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="203" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="204" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="205" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="206" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="207" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="208" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>